<commit_message>
fix: Costa Rica → Costa de Marfil (Grupo E) y corrección de datos
</commit_message>
<xml_diff>
--- a/data/resultados_reales.xlsx
+++ b/data/resultados_reales.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Fase Grupos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase Grupos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +100,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -122,11 +122,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -161,6 +205,8 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -526,7 +572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G89"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -556,6 +602,10 @@
           <t>AdminOficina</t>
         </is>
       </c>
+      <c r="D2" s="12" t="n"/>
+      <c r="E2" s="12" t="n"/>
+      <c r="F2" s="12" t="n"/>
+      <c r="G2" s="13" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="B3" s="4" t="inlineStr">
@@ -563,7 +613,13 @@
           <t>Rellena los goles previstos en cada partido. Fecha limite: 11 jun 2026 a las 17:00 h.</t>
         </is>
       </c>
-    </row>
+      <c r="C3" s="12" t="n"/>
+      <c r="D3" s="12" t="n"/>
+      <c r="E3" s="12" t="n"/>
+      <c r="F3" s="12" t="n"/>
+      <c r="G3" s="13" t="n"/>
+    </row>
+    <row r="4"/>
     <row r="5" ht="22" customHeight="1">
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -1234,7 +1290,7 @@
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Costa Rica 🇨🇷</t>
+          <t>Costa de Marfil 🇨🇮</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
@@ -1270,7 +1326,7 @@
       <c r="E37" s="9" t="n"/>
       <c r="F37" s="10" t="inlineStr">
         <is>
-          <t>🇨🇷 Costa Rica</t>
+          <t>🇨🇮 Costa de Marfil</t>
         </is>
       </c>
       <c r="G37" s="11" t="inlineStr">
@@ -1342,7 +1398,7 @@
       <c r="E40" s="9" t="n"/>
       <c r="F40" s="10" t="inlineStr">
         <is>
-          <t>🇨🇷 Costa Rica</t>
+          <t>🇨🇮 Costa de Marfil</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">

</xml_diff>

<commit_message>
auto: resultados 2026-06-12 07:32 UTC
</commit_message>
<xml_diff>
--- a/data/resultados_reales.xlsx
+++ b/data/resultados_reales.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fase Grupos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Fase Grupos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -670,8 +670,12 @@
           <t>G-A1-A2</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
+      <c r="D7" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
           <t>🇿🇦 Sudáfrica</t>
@@ -694,8 +698,12 @@
           <t>G-A3-A4</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
+      <c r="D8" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
           <t>🇨🇿 Chequia</t>

</xml_diff>

<commit_message>
auto: resultados 2026-06-13 04:46 UTC
</commit_message>
<xml_diff>
--- a/data/resultados_reales.xlsx
+++ b/data/resultados_reales.xlsx
@@ -1131,8 +1131,12 @@
           <t>G-D1-D2</t>
         </is>
       </c>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="D28" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E28" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="F28" s="10" t="inlineStr">
         <is>
           <t>🇵🇾 Paraguay</t>

</xml_diff>

<commit_message>
auto: resultados 2026-06-14 01:58 UTC
</commit_message>
<xml_diff>
--- a/data/resultados_reales.xlsx
+++ b/data/resultados_reales.xlsx
@@ -980,8 +980,12 @@
           <t>G-C1-C2</t>
         </is>
       </c>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
+      <c r="D21" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="F21" s="10" t="inlineStr">
         <is>
           <t>🇲🇦 Marruecos</t>

</xml_diff>

<commit_message>
auto: resultados 2026-06-14 06:37 UTC
</commit_message>
<xml_diff>
--- a/data/resultados_reales.xlsx
+++ b/data/resultados_reales.xlsx
@@ -1163,8 +1163,12 @@
           <t>G-D3-D4</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
+      <c r="D29" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>0</v>
+      </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
           <t>🇹🇷 Turquía</t>

</xml_diff>